<commit_message>
Daily facility note collection 2026-09-08
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D101"/>
+  <dimension ref="A1:D201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2638,6 +2638,2206 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>銀だこハイボール酒場 すすきのグルーヴビル店</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>https://stores.gindaco.com/detail/1011136/</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>9/11ザ・ビッグ厚別店</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g9V</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>赤から盛岡駅前通り店</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>https://akakara.jp/blogs/store-locator-menu/1815</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>ファミリーマート蔵王遠刈田店</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>https://www.family.co.jp/store.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>名前の無いパティスリー</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>https://tonomaruya.jp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>GOLDY ルミネ北千住店</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>https://goldy.jp/information</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>ELLE café TAKANAWA</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>https://ellecafe.jp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>MAKE UP FOR EVER そごう横浜店</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>https://www.sogo-seibu.jp/yokohama/brand/-make-up-for-ever</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Hangry Joe’s Tokyo 横浜中華街店</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>https://hangryjoestokyo.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>9/17明治屋自由が丘ストアー</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ga2</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>スーパーサウナ一宮</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>https://supersauna.jp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>立喰い寿司 魚椿 ミヤコ地下街店</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>https://shop.hikari-food-service.jp/stores</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>(9/8プレ)9/9スーパーセンタートライアル名張店</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2l</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>アイシティ そよら津桜橋店</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>https://www.eyecity.jp/shop/334/</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>(9/8ソフト)9/11そよら津桜橋(三重県津市)</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1bV2</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>JOYFULL EXPRESS イオンモール高知店</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>https://www.joyfull.co.jp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>9/1オーケー高槻赤大路店(大阪府高槻市)</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fOy</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>9/1 ライフ鎌倉梶原店</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fS5</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>9/3 サンディ吹田五月が丘店(大阪府吹田市)</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fPd</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>9/3改装 スーパーのアオキ直江津店(新潟県上越市)</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2v</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>9/3スギ薬局茜部南店(岐阜市)</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2N</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>9/4クックマート上西店（静岡県浜松市）</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7N</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>9/4(9/3プレ)スーパー生鮮館TAIGA桂子田店</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fZU</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>9/4改装 名古屋PARCO</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7c</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>9/4改装 メイチカ(名古屋市)</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7g</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>9/4ウルフギャングステーキハウス名古屋店</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eZr</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>9/4 ゴジラ・ストア Nagoya</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fn6</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>9/4ロピア彦根ナフコ店</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fNK</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>9/10改装 マルナカ檀紙店(香川県高松市)</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7X</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>9/10ザ・ビッグエクスプレスみよし店</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>9/10ファミリーマート中津川下野店</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g84</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>9/10とりせん田沼インター店(栃木県)</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g9g</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>9/11スーパーマーケットバロー豊中島江店</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fXN</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>9/16SANYO Style STORE PLUS イオンモール岡崎店</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fEw</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>9/17ロピア ムサシ新潟西店(新潟市)</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g6X</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>中国地方ハローズ呉広モール 2025年12月17日(水)開業！全7店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/42161</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>中部地方アークガレリア長岡 再開発 2026年春リニューアル完了！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/37232</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>関東地方みなとみらい21中央地区60・61街区開発事業 2029年春開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/36914</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>中国地方岩国駅前南地区市街地再開発事業 2030年春以降開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/24871</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>中部地方福井駅前南通り地区市街地再開発事業 2027年より順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/43036</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>北海道地方tonarie（トナリエ）北広島 2025年3月15日(土)開業！全テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/21566</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>関西地方オトカリテ跡地にイオンモールの大型商業施設 2027年以降開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/39391</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>関西地方【計画延期】大阪ガスビルディング（ガスビル） 再開発 2027年以降開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/30050</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>関東地方みと好文テラス 2026年4月23日(木)開業！全11テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48066</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>関西地方ヤマイチGARDEN桜井 マツゲンが出店！2025年11月21日(金)~順次開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/39875</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>関東地方赤坂二・六丁目地区開発計画 2028年秋完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/29750</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>関東地方ケーズデンキ厚木妻田東店 2027年春に開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47111</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>中部地方ロピアモール滝ノ水 2026年5月21日(木)開業！全7テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/48558</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>東北地方アスマチ多賀城 2025年10月着工！商業施設も！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/35915</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>九州地方OHASHI HILL ゆめアール大橋跡地に2025年4月18日(金)先行開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/27364</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>関東地方和光市駅北口地区市街地再開発事業 2029年度完成予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/32817</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>中部地方三郷駅前地区市街地再開発事業 2029年春完成予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/24605</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>関東地方カインズ伊勢崎境保泉店 2028年春開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47795</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>四国地方スーパーセンタートライアル松山空港通り店 2026年8月28日(金)グランドオープン！最新情報も！愛媛県松山市にトライアルカンパニーの店舗「スーパーセンタートライアル松山空港通り店」が2026年8月28日(金)グランドオープン！8月25日(火)～27日(木)プレオープン！スーパーセンタートライアルが松山市に初出店！そんな、スーパーセンタ...2026.09.08四国地方</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/shikoku/44917</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>関西地方ケーズデンキ桜井店 2026年9月17日(木)開業予定！最新情報も！奈良県桜井市に関西ケーズデンキの店舗「ケーズデンキ桜井店」が2026年9月17日(木)開業予定！ケーズデンキの大型店舗が、新たに誕生する桜井複合商業施設へ出店！隣接地にはコーナンPROも新設！そんな、ケーズデンキ桜井店について、テナントや開...2026.09.08関西地方</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/49275</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>アクロスプラザ高砂／兵庫県高砂市に9月9日オープン、マルアイ新業態も登場</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090819.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>ゆめマート熊本／「ゆめマート八代高田」9月14日、「ゆめマート九品寺」9月25日営業再開</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090811.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>ラゾーナ川崎／「月島もんじゃ くうや」10月3日オープン</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090817.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>俺のシリーズ／「俺の割烹 梅田北新地」9月7日オープン、和食ブランド関西初進出</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090814.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>ザボディショップ／さっぽろ東急百貨店にサステナブル店舗オープン、新幹線再生アルミを什器に活用</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090816.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>アルペン／山口県「おのだサンパーク」にスポーツデポ・ゴルフ5を9月11日同時オープン</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090813.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>マルキョウ／福岡市西区の「下山門店」9月22日閉店</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090815.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>トフロム八重洲 タワー／商業ゾーンに老舗や新業態など55店舗オープン、9月10日開業注目</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s090741.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>イオン／「イオンモール八千代緑が丘」9月18日リニューアル、ユニクロなど新規オープン</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090782.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>イオン九州／「マックスバリュ城栄店」9月10日オープン、ジョイフルサンを業態転換</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090774.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>三井不動産／津田沼PARCO跡地に駅前広場「ATOCHI」10月1日オープン</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090773.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>マムズタッチ／「新宿パークタワー店」オープン、日本法人オフィスを新宿に移転</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090777.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>資さんうどん／埼玉県本庄市に「児玉店」9月17日オープン、ガストを業態転換</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090778.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>まいばすけっと／千葉県鎌ケ谷市に「新鎌ヶ谷駅店」9月10日オープン</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090783.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>神戸屋／東武池袋駅構内にベーカリースタンド9月18日オープン、ドリンクも提供</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090711.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>猿田彦珈琲／皇居東御苑内に新店舗11月3日オープン</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090772.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>オリジン東秀／千葉県松戸市に「れんげ食堂Toshu 北小金店」9月9日オープン</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090712.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>すたみな太郎／青森県に「PREMIUM BUFFET弘前店」9月12日オープン、ベーカリー導入</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090775.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>イオンモール盛岡／屋内型こどもの遊び場「ちきゅうのにわ」10月7日オープン</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090713.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026年09月08日</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>ヨドバシカメラ／マルチメディア名鉄名古屋店9月16日オープン、総売場面積1万1900m2</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090484.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-09-09
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D201"/>
+  <dimension ref="A1:D301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4838,6 +4838,2206 @@
         </is>
       </c>
     </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>THE BODY SHOP さっぽろ東急百貨店</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>https://www.the-body-shop.co.jp/shop/e/ens260909/</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>キャトル・セゾン仙台</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>https://www.quatresaisons.co.jp/shop_list/id=176</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>https://www.fukudaya.net/event/6673</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>李暁七マーラータン</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>https://www.atre-kawagoe.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>BIZcomfort北赤羽</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>https://bizcomfort.jp/tokyo/kitaakabane.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>カデンシア＆コンシェル 玉川高島屋</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>https://www.takashimaya.co.jp/tamagawa/sc/departmentstore/topics/3_1_20260824132339/</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>弁才天 コレド室町テラス店</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>https://mitsui-shopping-park.com/urban/muromachi/information/index.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Arc’teryx 御殿場プレミアム・アウトレット店</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>https://www.premiumoutlets.co.jp/gotemba/brands/detail_1204.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>VAN 三越星が丘</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>https://www.van.co.jp/f/shoplist</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>RAW FUDGE ジェイアール名古屋タカシマヤ店</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>https://www.rawfudge.jp/news</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>9/9(9/8プレ)スーパーセンタートライアル名張店</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2l</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>BEIDELLI</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>https://www.hepfive.jp/newopen</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>コーナンPRO桜井店</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>https://kohnan-pro.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>デリカキッチン 大丸心斎橋店</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>https://chubufoods.co.jp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>富澤商店 宝塚阪急店</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>https://tomiz.com/store/detail/74</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>9/9MARUAI BIG アクロスプラザ高砂店</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gbn</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>アミュプラザ小倉 東館3階</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>https://www.amuplaza.jp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Green Cosmetic Garden 山形屋店</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>https://www.yamakataya.co.jp/kagoshima/news/</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>9/1オーケー高槻赤大路店(大阪府高槻市)</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fOy</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>9/1 ライフ鎌倉梶原店</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fS5</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>9/3 サンディ吹田五月が丘店(大阪府吹田市)</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fPd</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>9/3改装 スーパーのアオキ直江津店(新潟県上越市)</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2v</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>9/3スギ薬局茜部南店(岐阜市)</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2N</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>9/4クックマート上西店（静岡県浜松市）</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7N</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>9/4(9/3プレ)スーパー生鮮館TAIGA桂子田店</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fZU</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>9/4改装 名古屋PARCO</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7c</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>9/4改装 メイチカ(名古屋市)</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7g</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>9/4ウルフギャングステーキハウス名古屋店</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eZr</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>9/4 ゴジラ・ストア Nagoya</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fn6</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>9/4ロピア彦根ナフコ店</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fNK</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>(9/8ソフト)9/11そよら津桜橋(三重県津市)</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1bV2</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>9/10改装 マルナカ檀紙店(香川県高松市)</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7X</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>9/10ザ・ビッグエクスプレスみよし店</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>9/10ファミリーマート中津川下野店</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g84</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>9/10とりせん田沼インター店(栃木県)</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g9g</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>9/11スーパーマーケットバロー豊中島江店</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fXN</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>9/11ザ・ビッグ厚別店</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g9V</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>9/16SANYO Style STORE PLUS イオンモール岡崎店</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fEw</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>9/17ロピア ムサシ新潟西店(新潟市)</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g6X</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>9/17明治屋自由が丘ストアー</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ga2</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>関東地方フーコット多摩唐木田店 2027年1月開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47609</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>関東地方ニトリ宇都宮インターパーク店 2025年6月20日(金)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/40136</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>関東地方ヤオコー福生牛浜店 2026年1月20日(火)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42926</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>関東地方Beisia Foods Park 伊勢崎境保泉店 2028年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47770</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>関東地方ゆりストア百合丘本店 建て替え 2025年3月開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42337</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>中国地方エールエール広島 2026年3月5日(木) リニューアル開業！新規テナント16店舗出店！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/47002</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>関東地方ヤオコー大宮市場店 2026年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48511</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>関西地方そよら三田フラワータウン 2027年春開業！フローラ88 跡地 テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/39680</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>九州地方スーパーセンタートライアルうきは店 2026年11月下旬に開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/49325</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>関東地方イオンタウン小田原 2026年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/17418</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>関東地方そよら入曽駅前 2025年3月21日(金)開業！全テナント10店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/22304</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>関東地方明治安田新宿ビル 2026年11月下旬以降開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26240</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>関東地方アイタウン魚津 2025年10月16日(木)開業！無印良品も出店へ！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/43463</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>関東地方コトエ橋本 2026年5月29日(金)開業！全21テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/41085</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>中国地方ハローズ呉広モール 2025年12月17日(水)開業！全7店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/42161</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>北海道地方tonarie（トナリエ）北広島 2025年3月15日(土)開業！全テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/hokkaido/21566</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>関東地方グリーンシップタウン船橋 ブランズシティ船橋ビアレ 2028年12月開業！商業施設も誕生！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/34568</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>中部地方新潟駅万代口東地区開発計画 2028年夏開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/48895</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>四国地方スーパーセンタートライアル松山空港通り店 2026年8月28日(金)グランドオープン！最新情報も！愛媛県松山市にトライアルカンパニーの店舗「スーパーセンタートライアル松山空港通り店」が2026年8月28日(金)グランドオープン！8月25日(火)～27日(木)プレオープン！スーパーセンタートライアルが松山市に初出店！そんな、スーパーセンタ...2026.09.08四国地方</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/shikoku/44917</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>関西地方ケーズデンキ桜井店 2026年9月17日(木)開業予定！最新情報も！奈良県桜井市に関西ケーズデンキの店舗「ケーズデンキ桜井店」が2026年9月17日(木)開業予定！ケーズデンキの大型店舗が、新たに誕生する桜井複合商業施設へ出店！隣接地にはコーナンPROも新設！そんな、ケーズデンキ桜井店について、テナントや開...2026.09.08関西地方</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/49275</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>アットコスメストア／「ルミネ有楽町店」増床リニューアル、年間売上高11億円目指す注目</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s090973.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>アイン薬局／次世代型店舗「横浜南店」実験開始</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090913.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>平和堂／京都府城陽市に「（仮称）大久保店（店舗面積3805m2）」27年1月2日新設</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0909011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>コスモス薬品／大阪府和泉市に「ドラッグコスモスのぞみ野店」27年2月2日新設</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0909012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>ハンズ／東京都「自由が丘店」9月17日オープン、新施設「ミューズスクエア」に出店</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090950.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>スタバ／東名高速・浜名湖サービスエリア「ONE SEANA」に出店、9月18日オープン</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090946.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>物語コーポレーション／大阪府「寿司・しゃぶしゃぶ ゆず庵 堺鳳店」9月23日オープン</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090949.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>串カツ田中／京都市山科区に「椥辻店」オープン、新デザインの看板を採用</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090945.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>くすりのレデイ／兵庫県「東山店」、香川県「花ノ宮店」9月10日オープン</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090912.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>アクロスプラザ高砂／兵庫県高砂市に9月9日オープン、マルアイ新業態も登場</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090819.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>ゆめマート熊本／「ゆめマート八代高田」9月14日、「ゆめマート九品寺」9月25日営業再開</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090811.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>ラゾーナ川崎／「月島もんじゃ くうや」10月3日オープン</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090817.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>俺のシリーズ／「俺の割烹 梅田北新地」9月7日オープン、和食ブランド関西初進出</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090814.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>ザボディショップ／さっぽろ東急百貨店にサステナブル店舗オープン、新幹線再生アルミを什器に活用</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090816.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>アルペン／山口県「おのだサンパーク」にスポーツデポ・ゴルフ5を9月11日同時オープン</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090813.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>マルキョウ／福岡市西区の「下山門店」9月22日閉店</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090815.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>トフロム八重洲 タワー／商業ゾーンに老舗や新業態など55店舗オープン、9月10日開業注目</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s090741.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>イオン／「イオンモール八千代緑が丘」9月18日リニューアル、ユニクロなど新規オープン</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090782.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>イオン九州／「マックスバリュ城栄店」9月10日オープン、ジョイフルサンを業態転換</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090774.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>2026年09月09日</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>三井不動産／津田沼PARCO跡地に駅前広場「ATOCHI」10月1日オープン</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090773.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-09-10
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D301"/>
+  <dimension ref="A1:D397"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7038,6 +7038,2118 @@
         </is>
       </c>
     </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>9/10移転コープさっぽろ すながわ店</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fZi</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>とりせん田沼インター店(栃木県佐野市)</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g9g</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>9/10もとまちユニオン大船店</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gfg</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>9/10TOFROM YAESU TOWER(東京都中央区)</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ged</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>9/10ザ・ビッグエクスプレスみよし店</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>9/10ファミリーマート中津川下野店</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g84</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>9/10業務スーパー船場本町店</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gdW</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>9/10業務スーパー津山山北店</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ge1</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>9/10改装 マルナカ檀紙店(香川県高松市)</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7X</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>9/10ラ・ムー飯塚花瀬店(福岡県飯塚市)</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ge8</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>9/10改装マックスバリュ城栄店(長崎市)</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gel</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>9/1オーケー高槻赤大路店(大阪府高槻市)</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fOy</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>9/1 ライフ鎌倉梶原店</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fS5</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>9/3 サンディ吹田五月が丘店(大阪府吹田市)</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fPd</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>9/3改装 スーパーのアオキ直江津店(新潟県上越市)</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2v</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>9/3スギ薬局茜部南店(岐阜市)</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2N</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>9/4クックマート上西店（静岡県浜松市）</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7N</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>9/4(9/3プレ)スーパー生鮮館TAIGA桂子田店</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fZU</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>9/4改装 名古屋PARCO</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7c</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>9/4改装 メイチカ(名古屋市)</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7g</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>9/4ウルフギャングステーキハウス名古屋店</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eZr</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>9/4 ゴジラ・ストア Nagoya</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fn6</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>9/4ロピア彦根ナフコ店</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fNK</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>(9/8ソフト)9/11そよら津桜橋(三重県津市)</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1bV2</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>9/9MARUAI BIG アクロスプラザ高砂店</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gbn</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>9/11スーパーマーケットバロー豊中島江店</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fXN</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>9/11ザ・ビッグ厚別店</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g9V</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>9/16SANYO Style STORE PLUS イオンモール岡崎店</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fEw</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>9/17ロピア ムサシ新潟西店(新潟市)</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g6X</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>9/17明治屋自由が丘ストアー</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ga2</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>関東地方プラウドタワー板橋 2027年秋開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26709</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>中部地方イータウン大広田 2025年5月28日(水)開業！全テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/40691</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>九州地方ゆめモール那珂川 2026年2月20日(金)~順次開業！全20店舗一覧！</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/31176</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>中国地方岩国駅前南地区市街地再開発事業 2030年春以降開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/24871</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>中部地方スーパーセンタートライアル名古屋みなと店 2026年11月開業予定！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/48009</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>関東地方イオンモール津田沼サウス 2026年3月18日(水)開業！全50店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/45209</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>関東地方新横浜プリンスペペ 2027年3月閉店の理由は？跡地はマクニカ新社屋に！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47961</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>関東地方イオン新座店 2024年2月29日(木)に閉店し建て替えて2027年度開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/36881</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>九州地方レイリア春日原 2026年6月11日(木)開業！全10店舗一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/38672</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>関東地方エキュート秋葉原 2025年4月7日(月)10時~開業！全24テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/42906</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>中部地方名古屋ちゃやまちモール ロピア名古屋茶屋 2026年1月29日(木)10：00~開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/42218</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>関東地方立石駅北口地区市街地再開発事業 2030年春完成予定！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/21472</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>四国地方イオン坂出店 2024年2月29日(木)に閉店し建て替えへ！跡地はどうなる？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/shikoku/34197</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>九州地方ニトリ熊本はません店 2026年7月31日(金)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/48407</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>九州地方天神ブリッククロス 2025年4月竣工！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/22763</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>関東地方大山町ピッコロ・スクエア周辺地区市街地再開発事業 2030年度完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26424</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>関東地方アイタウン魚津 2025年10月16日(木)開業！無印良品も出店へ！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/43463</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>関東地方中山駅南口地区市街地再開発事業 2029年度完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/26880</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>中部地方マックスバリュ豊橋西幸町店 2027年春開業！テナントは？最新情報も！愛知県豊橋市西幸町に、食品スーパーマーケットを中心とした商業施設「(仮称)マックスバリュ豊橋西幸町店」が2027年4月頃にオープン予定！「愛知経済連豊橋食肉センター」の跡地約1.5万㎡を活用！マックスバリュ東海による豊橋市内4店舗目の出店と...2026.09.09中部地方</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/48626</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>関東地方ザ・マーケットプレイス綾瀬 カインズやケーズデンキ 2027年度出店へ！最新情報も！神奈川県綾瀬市の旧消防本部庁舎跡地および旧綾瀬タウンヒルズSC跡地に、ヤオコー主導の大型商業施設群「ザ・マーケットプレイス綾瀬」が誕生！旧消防本部跡地（北エリア）に「ヤオコー綾瀬店」と「ユニクロ」が先行開業！さらに2025年2月に閉館した綾...2026.09.09関東地方</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/29762</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>平和堂／「アルプラフーズマーケット富山掛尾」オープン、富山県に食品スーパー初出店</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091042.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>二子玉川ライズS.C.／今秋「マリークワント」「プリンセスタルト」など新規オープン</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091077.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>グランベリーパーク／秋リニューアルを実施、ラベンハムなど12店舗がオープン</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091045.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>DNP／グランスタ東京にブランド体験型店舗「＆found」今冬オープン</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091013.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>ヨドバシカメラ／東京・池袋に「リカーワールド ヨドバシ池袋店」9月19日オープン</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091044.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>まいばすけっと／神奈川県藤沢市に「湘南台駅西店」9月11日オープン</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091071.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>ニトリ／東京・神奈川の島忠2店舗にレディスアパレル「N+」9月11日オープン</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091072.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>ジョイフル本田／都内にペット専門店「Pet’s CLOVER東久留米南町店」12月オープン</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091074.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>イオンペット／山口県「ペテモおのだサンパーク店」9月11日オープン</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091073.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>コスモス薬品／岡山県・静岡県に「ドラッグコスモス」計2店舗、27年3月新設</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0910012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>クスリのアオキ／宮城県大崎市に「古川旭店」27年2月16日新設</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0910011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>アットコスメストア／「ルミネ有楽町店」増床リニューアル、年間売上高11億円目指す注目</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/report/s090973.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>アイン薬局／次世代型店舗「横浜南店」実験開始</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090913.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>平和堂／京都府城陽市に「（仮称）大久保店（店舗面積3805m2）」27年1月2日新設</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0909011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>コスモス薬品／大阪府和泉市に「ドラッグコスモスのぞみ野店」27年2月2日新設</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0909012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>ハンズ／東京都「自由が丘店」9月17日オープン、新施設「ミューズスクエア」に出店</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090950.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>スタバ／東名高速・浜名湖サービスエリア「ONE SEANA」に出店、9月18日オープン</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090946.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>物語コーポレーション／大阪府「寿司・しゃぶしゃぶ ゆず庵 堺鳳店」9月23日オープン</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090949.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>串カツ田中／京都市山科区に「椥辻店」オープン、新デザインの看板を採用</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090945.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>2026年09月10日</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>くすりのレデイ／兵庫県「東山店」、香川県「花ノ宮店」9月10日オープン</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s090912.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-09-11
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D397"/>
+  <dimension ref="A1:D487"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9150,6 +9150,1986 @@
         </is>
       </c>
     </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>9/11改装 ザ・ビッグ厚別店</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g9V</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>9/11Beisia Foods Park 岐南店</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gg7</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>9/1オーケー高槻赤大路店(大阪府高槻市)</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fOy</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>9/1 ライフ鎌倉梶原店</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fS5</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>9/3 サンディ吹田五月が丘店(大阪府吹田市)</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fPd</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>9/3改装 スーパーのアオキ直江津店(新潟県上越市)</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2v</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>9/3スギ薬局茜部南店(岐阜市)</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2N</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>9/4クックマート上西店（静岡県浜松市）</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7N</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>9/4(9/3プレ)スーパー生鮮館TAIGA桂子田店</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fZU</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>9/4改装 名古屋PARCO</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7c</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>9/4改装 メイチカ(名古屋市)</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7g</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>9/4ウルフギャングステーキハウス名古屋店</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eZr</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>9/4 ゴジラ・ストア Nagoya</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fn6</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>9/4ロピア彦根ナフコ店</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fNK</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>(9/8ソフト)9/11そよら津桜橋(三重県津市)</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1bV2</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>9/9MARUAI BIG アクロスプラザ高砂店</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gbn</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>9/10改装 マルナカ檀紙店(香川県高松市)</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7X</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>9/10ザ・ビッグエクスプレスみよし店</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>9/10ファミリーマート中津川下野店</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g84</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>9/10とりせん田沼インター店(栃木県)</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g9g</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>9/11スーパーマーケットバロー豊中島江店</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fXN</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>9/16SANYO Style STORE PLUS イオンモール岡崎店</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fEw</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>9/17ロピア ムサシ新潟西店(新潟市)</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g6X</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>9/17明治屋自由が丘ストアー</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ga2</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>東北地方イオン仙台店 跡地に複合ビル建設へ 2029年度開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/40539</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>九州地方トライアルスマート東長崎店 2025年8月20日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/42038</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>関西地方iyouTown（アイユータウン）須磨 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/43508</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>東北地方イオンタウン 福島市南矢野目に進出！2028年10月開業！ テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/38134</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>九州地方天神ブリッククロス 2025年4月竣工！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/22763</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>関西地方ハローズ洲本モール 2026年冬開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/42115</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>関東地方伊勢崎境ショッピングパーク 2027年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47294</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>関西地方平和堂岸辺店 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/49465</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>関西地方そよら小野 2027年秋開業！イオン小野店跡地 21店舗が出店！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/43512</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>関西地方ハローズ本多聞店 2026年6月24日(水)から順次開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/46204</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>九州地方キャナルシティ博多イーストビル 2026年9月4日(金)開業！全16店舗一覧！</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/30939</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>関東地方アークタウン宇都宮 2026年3月28日(土)開業！全5テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47363</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>中国地方スーパーセンタートライアル大田店 2025年6月18日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/40704</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>九州地方糸満市真栄里地区商業施設 2028年開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kyushu/47815</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>関東地方品川駅北口に新駅ビル 2031年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/33951</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>中部地方ベイシア長久手店 2025年3月5日(水)開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/38015</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>関東地方桜川ショッピングセンター(仮称) 2027年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/34191</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>関東地方アイタウン魚津 2025年10月16日(木)開業！無印良品も出店へ！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/43463</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>関西地方平和堂大久保店 2027年春開業！テナントは？最新情報も！京都府城陽市平川（旧24号線沿い・旧イズミヤ大久保店跡地）に、大手スーパー・株式会社平和堂による大型複合スーパーマーケット「(仮称)平和堂大久保店」が2027年春開業予定！約52年間にわたり城陽・大久保エリアの生活拠点として親しまれ、202...2026.09.10関西地方</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/49605</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>関東地方東京ミッドタウン日本橋 2027年秋開業！コレド日本橋も大規模改装！テナントは？最新情報も！東京都中央区日本橋のコレド日本橋隣接地に建設中の、三井不動産や野村不動産などが手掛ける超高層再開発ビル「東京ミッドタウン日本橋」が2026年9月末に竣工し、2027年秋にグランドオープンします！これまで「日本橋一丁目中地区市街地再開発事業」...2026.09.10関東地方</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/17615</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>ヤオコー／千葉県船橋市に「船橋薬円台店」9月15日オープン</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091116.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>バロー／名古屋市に「スーパーマーケットバロー矢田店」9月18日オープン</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091115.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>ベイシア／三心との連携1号店「岐南店」改装オープン、即食品強化・丸魚の販売継続</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091172.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>池袋パルコ／大規模リニューアル完了「ウルトラマンストア」など今秋15店舗オープン</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091176.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>仙台パルコ／秋冬リニューアルで新規含む16店舗オープン、PARCO2では飲食強化</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091175.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>あべのハルカス近鉄本店／10～11月、子ども服フロアの大規模リニューアル開始</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091114.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>コスモス薬品／福岡県・島根県に「ドラッグコスモス」計2店舗、27年4月新設</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0911012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>ビームス／原宿に「ビームス レコーズ／bPrビームス」9月19日オープン</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091113.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>フライングタイガー／池袋・サンシャインシティに10月16日新店舗オープン</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091112.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>JR西日本／大阪駅にメーク直し・仕事・休憩に対応する駅ナカ空間オープン</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091118.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>成城石井／大阪府守口市に「京阪百貨店守口店」10月8日オープン</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091141.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>オンデーズ／三重県4店舗目「OWNDAYS そよら津桜橋店」オープン</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091177.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>ケーズデンキ／宮城県名取市に「（仮称）新仙台南店（店舗面積5988.15m2）」27年3月23日新設</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0911011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>平和堂／「アルプラフーズマーケット富山掛尾」オープン、富山県に食品スーパー初出店</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091042.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>二子玉川ライズS.C.／今秋「マリークワント」「プリンセスタルト」など新規オープン</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091077.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>グランベリーパーク／秋リニューアルを実施、ラベンハムなど12店舗がオープン</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091045.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>DNP／グランスタ東京にブランド体験型店舗「＆found」今冬オープン</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091013.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>ヨドバシカメラ／東京・池袋に「リカーワールド ヨドバシ池袋店」9月19日オープン</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091044.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>まいばすけっと／神奈川県藤沢市に「湘南台駅西店」9月11日オープン</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091071.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>2026年09月11日</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>ニトリ／東京・神奈川の島忠2店舗にレディスアパレル「N+」9月11日オープン</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091072.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-09-12
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D487"/>
+  <dimension ref="A1:D576"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11130,6 +11130,1964 @@
         </is>
       </c>
     </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>9/1オーケー高槻赤大路店(大阪府高槻市)</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fOy</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>9/1 ライフ鎌倉梶原店</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fS5</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>9/3 サンディ吹田五月が丘店(大阪府吹田市)</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fPd</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>9/3改装 スーパーのアオキ直江津店(新潟県上越市)</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2v</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>9/3スギ薬局茜部南店(岐阜市)</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2N</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>9/4クックマート上西店（静岡県浜松市）</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7N</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>9/4(9/3プレ)スーパー生鮮館TAIGA桂子田店</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fZU</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>9/4改装 名古屋PARCO</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7c</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>9/4改装 メイチカ(名古屋市)</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7g</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>9/4ウルフギャングステーキハウス名古屋店</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eZr</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>9/4 ゴジラ・ストア Nagoya</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fn6</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>9/4ロピア彦根ナフコ店</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fNK</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>(9/8ソフト)9/11そよら津桜橋(三重県津市)</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1bV2</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>9/9MARUAI BIG アクロスプラザ高砂店</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1gbn</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>9/10改装 マルナカ檀紙店(香川県高松市)</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7X</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>9/10ザ・ビッグエクスプレスみよし店</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>9/10ファミリーマート中津川下野店</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g84</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>9/10とりせん田沼インター店(栃木県)</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g9g</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>9/11スーパーマーケットバロー豊中島江店</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fXN</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>9/11ザ・ビッグ厚別店</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g9V</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>9/16SANYO Style STORE PLUS イオンモール岡崎店</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fEw</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>9/17ロピア ムサシ新潟西店(新潟市)</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g6X</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>9/17明治屋自由が丘ストアー</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1ga2</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>関西地方そよら三田フラワータウン 2027年春開業！フローラ88 跡地 テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/39680</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>関東地方秋葉原UDX アキバイチが2026年1月23日(金) 閉店 2026年冬リニューアル開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/46578</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>四国地方スーパーセンタートライアル三木店 2025年7月16日(水)開業！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/shikoku/41508</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>関東地方竹ノ塚駅東口地区市街地再開発事業 2035年以降開業！どのような施設になる？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48886</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>中国地方イオンタウン大田が増床！2025年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/40837</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>関西地方プリコ西明石 南館 2026年6月26日(金)開業！全6テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/42350</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>関東地方【第2六本木ヒルズ】六本木五丁目西地区市街地再開発事業 2030年度開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/33812</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>関東地方道玄坂二丁目南地区市街地再開発事業 2027年春開業予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/23396</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>関東地方JR武蔵境駅東側開発 2028年開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48480</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>関西地方イオンタウン平野跡地に商業施設 2027年冬開業！ テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/42949</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>中部地方コストコ亀山倉庫店 2028年以降開業！場所は？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/23805</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>関東地方つくば市陣場複合施設 2027年春開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/49177</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>関西地方茶屋町B-2・B-3地区市街地再開発事業 2028年度完成予定！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/29719</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>関東地方北青山三丁目地区市街地再開発事業 2030年竣工！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/48749</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>中部地方イオンスタイル諏訪 2026年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chubu/36918</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>中国地方【呉駅前再開発】呉駅周辺地域総合開発事業 2027年度開業！どのような施設に？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/chugoku/26750</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>関東地方ベルク平塚田村店 2026年秋開業！テナントは？最新情報も！</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47482</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>関東地方アークタウン宇都宮 2026年3月28日(土)開業！全5テナント一覧！最新情報も！</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kantou/47363</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>関西地方ケーズデンキ桜井店 2026年9月17日(木)開業予定！最新情報も！奈良県桜井市に関西ケーズデンキの店舗「ケーズデンキ桜井店」が2026年9月17日(木)開業予定！ケーズデンキの大型店舗が、新たに誕生する桜井複合商業施設へ出店！隣接地にはコーナンPROも新設！そんな、ケーズデンキ桜井店について、テナントや開...2026.09.12関西地方</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/kansai/49275</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>出店ウォッチ</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>東北地方スーパーセンタートライアル金ケ崎店 2026年9月16日(水)開業！15日(火)プレオープン！最新情報も！岩手県胆沢郡金ケ崎町にトライアルカンパニーの店舗「スーパーセンタートライアル金ケ崎店」が2026年9月16日(水)8：30グランドオープン！9月15日(火)10：00～19：00プレオープン！スーパーセンタートライアルが金ケ崎町に初出店！そ...2026.09.12東北地方</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>https://shutten-watch.com/touhoku/47232</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>ヤオコー／千葉県船橋市に「船橋薬円台店」9月15日オープン</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091116.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>バロー／名古屋市に「スーパーマーケットバロー矢田店」9月18日オープン</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091115.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>ベイシア／三心との連携1号店「岐南店」改装オープン、即食品強化・丸魚の販売継続</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091172.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>池袋パルコ／大規模リニューアル完了「ウルトラマンストア」など今秋15店舗オープン</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091176.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>仙台パルコ／秋冬リニューアルで新規含む16店舗オープン、PARCO2では飲食強化</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091175.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>あべのハルカス近鉄本店／10～11月、子ども服フロアの大規模リニューアル開始</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091114.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>コスモス薬品／福岡県・島根県に「ドラッグコスモス」計2店舗、27年4月新設</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0911012.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>ビームス／原宿に「ビームス レコーズ／bPrビームス」9月19日オープン</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091113.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>フライングタイガー／池袋・サンシャインシティに10月16日新店舗オープン</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091112.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>JR西日本／大阪駅にメーク直し・仕事・休憩に対応する駅ナカ空間オープン</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091118.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>成城石井／大阪府守口市に「京阪百貨店守口店」10月8日オープン</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091141.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>オンデーズ／三重県4店舗目「OWNDAYS そよら津桜橋店」オープン</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091177.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>ケーズデンキ／宮城県名取市に「（仮称）新仙台南店（店舗面積5988.15m2）」27年3月23日新設</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s0911011.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>平和堂／「アルプラフーズマーケット富山掛尾」オープン、富山県に食品スーパー初出店</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091042.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>二子玉川ライズS.C.／今秋「マリークワント」「プリンセスタルト」など新規オープン</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091077.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>グランベリーパーク／秋リニューアルを実施、ラベンハムなど12店舗がオープン</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091045.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>DNP／グランスタ東京にブランド体験型店舗「＆found」今冬オープン</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091013.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>ヨドバシカメラ／東京・池袋に「リカーワールド ヨドバシ池袋店」9月19日オープン</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091044.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>まいばすけっと／神奈川県藤沢市に「湘南台駅西店」9月11日オープン</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091071.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>2026年09月12日</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>流通ニュース</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>ニトリ／東京・神奈川の島忠2店舗にレディスアパレル「N+」9月11日オープン</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>https://www.ryutsuu.biz/store/s091072.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>